<commit_message>
chore(data): archive RGI 荣誉勋章(83人天) + 小美龙再生邮局(65人天) + index/history 自学习更新
- RGI 荣誉勋章_20260915: 83 人天基准 + 102/50 报价版 + Medtronic 客户报价单
- 小美龙再生邮局_20260915: 65 人天（自营库存+预约到店口径，含 v7 手改同步）
- Facility 三期需求估算.xlsx: 手改同步入库
- 库状态: 16 项目 / 330 feature / 24 种功能模式均有实例
</commit_message>
<xml_diff>
--- a/data/estimations/Facility 三期需求_20260909/Facility 三期需求估算.xlsx
+++ b/data/estimations/Facility 三期需求_20260909/Facility 三期需求估算.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaoming\workspace\project-effort-estimation\data\current\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaoming\workspace\project-effort-estimation\data\estimations\Facility 三期需求_20260909\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12255"/>
+    <workbookView windowWidth="28800" windowHeight="12975"/>
   </bookViews>
   <sheets>
     <sheet name="工时估算" sheetId="1" r:id="rId1"/>
@@ -130,7 +130,7 @@
     <t>工单数据统计看板与报告导出（含工单评价统计）</t>
   </si>
   <si>
-    <t>统计看板（工单量趋势/状态/类型/处理时效+评价汇总）6、报告导出Excel 1</t>
+    <t xml:space="preserve">统计看板（工单量趋势/状态/类型/处理时效+评价汇总）、报告导出Excel </t>
   </si>
   <si>
     <t>评论支持图片</t>
@@ -1378,16 +1378,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
+  <dimension ref="A1:I39"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="5.70833333333333" customWidth="1"/>
     <col min="2" max="2" width="15.7083333333333" customWidth="1"/>
     <col min="3" max="3" width="30.7083333333333" customWidth="1"/>
     <col min="4" max="4" width="12.375" customWidth="1"/>
     <col min="5" max="5" width="40.7083333333333" customWidth="1"/>
-    <col min="6" max="6" width="10.7083333333333" customWidth="1"/>
-    <col min="7" max="7" width="12.7083333333333" customWidth="1"/>
+    <col min="6" max="6" width="10.7083333333333" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="10.875" customWidth="1"/>
     <col min="8" max="8" width="30.7083333333333" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1721,7 +1721,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" s="2">
         <v>11</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="18" ht="27" spans="1:8">
+    <row r="18" ht="27" spans="1:9">
       <c r="A18" s="2">
         <v>12</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" ht="27" spans="1:8">
+    <row r="19" ht="27" spans="1:9">
       <c r="A19" s="2">
         <v>13</v>
       </c>
@@ -1788,8 +1788,11 @@
       <c r="H19" s="3" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" ht="27" spans="1:8">
+      <c r="I19">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" ht="27" spans="1:9">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="3"/>
@@ -1805,7 +1808,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="21" ht="67.5" spans="1:8">
+    <row r="21" ht="67.5" spans="1:9">
       <c r="A21" s="2">
         <v>14</v>
       </c>
@@ -1826,8 +1829,11 @@
       <c r="H21" s="3" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="22" ht="40.5" spans="1:8">
+      <c r="I21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" ht="40.5" spans="1:9">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="3"/>
@@ -1843,7 +1849,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" ht="121.5" spans="1:8">
+    <row r="23" ht="121.5" spans="1:9">
       <c r="A23" s="2">
         <v>15</v>
       </c>
@@ -1864,8 +1870,11 @@
       <c r="H23" s="3" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="24" ht="81" spans="1:8">
+      <c r="I23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" ht="81" spans="1:9">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="3"/>
@@ -1883,7 +1892,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" ht="94.5" spans="1:8">
+    <row r="25" ht="94.5" spans="1:9">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="3"/>
@@ -1901,7 +1910,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" ht="27" spans="1:8">
+    <row r="26" ht="27" spans="1:9">
       <c r="A26" s="2">
         <v>16</v>
       </c>
@@ -1922,8 +1931,11 @@
       <c r="H26" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="27" ht="40.5" spans="1:8">
+      <c r="I26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" ht="40.5" spans="1:9">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="3"/>
@@ -1939,7 +1951,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" ht="27" spans="1:8">
+    <row r="28" ht="27" spans="1:9">
       <c r="A28" s="2">
         <v>17</v>
       </c>
@@ -1960,8 +1972,11 @@
       <c r="H28" s="3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="29" spans="1:8">
+      <c r="I28">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" s="2">
         <v>18</v>
       </c>
@@ -1982,7 +1997,7 @@
       </c>
       <c r="H29" s="3"/>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:9">
       <c r="A30" s="2">
         <v>19</v>
       </c>
@@ -2002,7 +2017,7 @@
       </c>
       <c r="H30" s="3"/>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:9">
       <c r="A31" s="2">
         <v>20</v>
       </c>
@@ -2022,7 +2037,7 @@
       </c>
       <c r="H31" s="3"/>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:9">
       <c r="A32" s="2">
         <v>21</v>
       </c>
@@ -2057,7 +2072,7 @@
       </c>
       <c r="H33" s="6"/>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" hidden="1" spans="1:8">
       <c r="A36" s="8" t="s">
         <v>84</v>
       </c>
@@ -2067,7 +2082,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" hidden="1" spans="1:8">
       <c r="A37" s="11" t="s">
         <v>86</v>
       </c>
@@ -2077,7 +2092,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" hidden="1" spans="1:8">
       <c r="A38" s="11" t="s">
         <v>88</v>
       </c>
@@ -2087,7 +2102,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" hidden="1" spans="1:8">
       <c r="A39" s="11" t="s">
         <v>90</v>
       </c>

</xml_diff>